<commit_message>
Wire in 14th Lane Urban Hotel + Marlborough Lodge geni.us links (Blenheim)
</commit_message>
<xml_diff>
--- a/Bryant_Jonathan_NZ_32Days_CRM.xlsx
+++ b/Bryant_Jonathan_NZ_32Days_CRM.xlsx
@@ -3005,17 +3005,13 @@
           <t>14th Lane Urban Hotel</t>
         </is>
       </c>
-      <c r="E88" t="inlineStr"/>
-      <c r="F88" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G88" t="inlineStr">
-        <is>
-          <t>⚠ Link to confirm</t>
-        </is>
-      </c>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>https://geni.us/14LaneBlenheim</t>
+        </is>
+      </c>
+      <c r="F88" t="inlineStr"/>
+      <c r="G88" t="inlineStr"/>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
@@ -3038,17 +3034,13 @@
           <t>Marlborough Lodge</t>
         </is>
       </c>
-      <c r="E89" t="inlineStr"/>
-      <c r="F89" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G89" t="inlineStr">
-        <is>
-          <t>⚠ Link to confirm</t>
-        </is>
-      </c>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>https://geni.us/MarlboroughLodge</t>
+        </is>
+      </c>
+      <c r="F89" t="inlineStr"/>
+      <c r="G89" t="inlineStr"/>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">

</xml_diff>

<commit_message>
Fiordland: 8 Apr Doubtful Sound Overnight Cruise, return 9 Apr + 2 nights Te Anau
</commit_message>
<xml_diff>
--- a/Bryant_Jonathan_NZ_32Days_CRM.xlsx
+++ b/Bryant_Jonathan_NZ_32Days_CRM.xlsx
@@ -425,16 +425,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G211"/>
+  <dimension ref="A1:G210"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
-    <col width="42" customWidth="1" min="2" max="2"/>
+    <col width="44" customWidth="1" min="2" max="2"/>
     <col width="22" customWidth="1" min="3" max="3"/>
-    <col width="52" customWidth="1" min="4" max="4"/>
+    <col width="54" customWidth="1" min="4" max="4"/>
     <col width="34" customWidth="1" min="5" max="5"/>
     <col width="9" customWidth="1" min="6" max="6"/>
-    <col width="34" customWidth="1" min="7" max="7"/>
+    <col width="40" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -4508,26 +4508,30 @@
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>Wanaka → Te Anau (via Queenstown)</t>
+          <t>Wanaka → Doubtful Sound Overnight Cruise (via Queenstown)</t>
         </is>
       </c>
       <c r="C140" t="inlineStr">
         <is>
-          <t>✨ Special Activity</t>
+          <t>🚢 Overnight Cruise</t>
         </is>
       </c>
       <c r="D140" t="inlineStr">
         <is>
-          <t>RealNZ Doubtful Sound Wilderness Cruise</t>
+          <t>Doubtful Sound Overnight Cruise (overnight aboard) — RealNZ</t>
         </is>
       </c>
       <c r="E140" t="inlineStr">
         <is>
-          <t>https://geni.us/DoubtfulDayTour</t>
+          <t>https://geni.us/DoubtfulOvernight</t>
         </is>
       </c>
       <c r="F140" t="inlineStr"/>
-      <c r="G140" t="inlineStr"/>
+      <c r="G140" t="inlineStr">
+        <is>
+          <t>Confirmed · board Manapouri 8 Apr, return midday 9 Apr</t>
+        </is>
+      </c>
     </row>
     <row r="141">
       <c r="A141" t="inlineStr">
@@ -4595,51 +4599,55 @@
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>Wanaka → Te Anau (via Queenstown)</t>
+          <t>Wanaka → Doubtful Sound Overnight Cruise (via Queenstown)</t>
         </is>
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t>🏡 Accommodation (3★)</t>
+          <t>🏡 Accommodation</t>
         </is>
       </c>
       <c r="D143" t="inlineStr">
         <is>
-          <t>Annies on Milford</t>
+          <t>Aboard Doubtful Sound Overnight Cruise — not in Te Anau</t>
         </is>
       </c>
       <c r="E143" t="inlineStr">
         <is>
-          <t>https://geni.us/AnniesTeAnau</t>
+          <t>https://geni.us/DoubtfulOvernight</t>
         </is>
       </c>
       <c r="F143" t="inlineStr"/>
-      <c r="G143" t="inlineStr"/>
+      <c r="G143" t="inlineStr">
+        <is>
+          <t>Overnight aboard</t>
+        </is>
+      </c>
     </row>
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>Thu 8 Apr</t>
+          <t>Fri 9 Apr</t>
         </is>
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>Wanaka → Te Anau (via Queenstown)</t>
+          <t>Fiordland – Te Anau (2 nights · 9–10 Apr)</t>
         </is>
       </c>
       <c r="C144" t="inlineStr">
         <is>
-          <t>🏡 Accommodation (4★)</t>
+          <t>🏡 Accommodation (3★)</t>
         </is>
       </c>
       <c r="D144" t="inlineStr">
         <is>
-          <t>Dusky Ridges</t>
+          <t>Annies on Milford</t>
         </is>
       </c>
       <c r="E144" t="inlineStr">
         <is>
-          <t>https://geni.us/DuskyRidges</t>
+          <t>https://geni.us/AnniesTeAnau</t>
         </is>
       </c>
       <c r="F144" t="inlineStr"/>
@@ -4648,27 +4656,27 @@
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>Thu 8 Apr</t>
+          <t>Fri 9 Apr</t>
         </is>
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>Wanaka → Te Anau (via Queenstown)</t>
+          <t>Fiordland – Te Anau (2 nights · 9–10 Apr)</t>
         </is>
       </c>
       <c r="C145" t="inlineStr">
         <is>
-          <t>🏡 Accommodation (5★)</t>
+          <t>🏡 Accommodation (4★)</t>
         </is>
       </c>
       <c r="D145" t="inlineStr">
         <is>
-          <t>Fiordland Lodge</t>
+          <t>Dusky Ridges</t>
         </is>
       </c>
       <c r="E145" t="inlineStr">
         <is>
-          <t>https://geni.us/FiordlandLodge</t>
+          <t>https://geni.us/DuskyRidges</t>
         </is>
       </c>
       <c r="F145" t="inlineStr"/>
@@ -4682,22 +4690,22 @@
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>Fiordland – Milford Sound</t>
+          <t>Fiordland – Te Anau (2 nights · 9–10 Apr)</t>
         </is>
       </c>
       <c r="C146" t="inlineStr">
         <is>
-          <t>✨ Special Activity</t>
+          <t>🏡 Accommodation (5★)</t>
         </is>
       </c>
       <c r="D146" t="inlineStr">
         <is>
-          <t>Trips &amp; Tramps – Milford Cruise &amp; Walk</t>
+          <t>Fiordland Lodge</t>
         </is>
       </c>
       <c r="E146" t="inlineStr">
         <is>
-          <t>https://geni.us/TripsTrampsMilford</t>
+          <t>https://geni.us/FiordlandLodge</t>
         </is>
       </c>
       <c r="F146" t="inlineStr"/>
@@ -4721,12 +4729,12 @@
       </c>
       <c r="D147" t="inlineStr">
         <is>
-          <t>T&amp;T Milford Track Guided Day Walk &amp; Cruise</t>
+          <t>Trips &amp; Tramps – Milford Cruise &amp; Walk</t>
         </is>
       </c>
       <c r="E147" t="inlineStr">
         <is>
-          <t>https://geni.us/TripsTrampsMilfordWalk</t>
+          <t>https://geni.us/TripsTrampsMilford</t>
         </is>
       </c>
       <c r="F147" t="inlineStr"/>
@@ -4750,12 +4758,12 @@
       </c>
       <c r="D148" t="inlineStr">
         <is>
-          <t>Fiordland Helicopters Scenic Flight</t>
+          <t>T&amp;T Milford Track Guided Day Walk &amp; Cruise</t>
         </is>
       </c>
       <c r="E148" t="inlineStr">
         <is>
-          <t>https://geni.us/FiordlandHelicopters</t>
+          <t>https://geni.us/TripsTrampsMilfordWalk</t>
         </is>
       </c>
       <c r="F148" t="inlineStr"/>
@@ -4779,12 +4787,12 @@
       </c>
       <c r="D149" t="inlineStr">
         <is>
-          <t>Milford Sound Overnight Cruise</t>
+          <t>Fiordland Helicopters Scenic Flight</t>
         </is>
       </c>
       <c r="E149" t="inlineStr">
         <is>
-          <t>https://geni.us/MilfordOvernighter</t>
+          <t>https://geni.us/FiordlandHelicopters</t>
         </is>
       </c>
       <c r="F149" t="inlineStr"/>
@@ -4793,12 +4801,12 @@
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>Sat 10 Apr</t>
+          <t>Fri 9 Apr</t>
         </is>
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>Fiordland – Doubtful Sound &amp; Kepler</t>
+          <t>Fiordland – Milford Sound</t>
         </is>
       </c>
       <c r="C150" t="inlineStr">
@@ -4808,12 +4816,12 @@
       </c>
       <c r="D150" t="inlineStr">
         <is>
-          <t>RealNZ Doubtful Sound Wilderness Day Cruise</t>
+          <t>Milford Sound Overnight Cruise</t>
         </is>
       </c>
       <c r="E150" t="inlineStr">
         <is>
-          <t>https://geni.us/DoubtfulDayTour</t>
+          <t>https://geni.us/MilfordOvernighter</t>
         </is>
       </c>
       <c r="F150" t="inlineStr"/>
@@ -4827,7 +4835,7 @@
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>Fiordland – Doubtful Sound &amp; Kepler</t>
+          <t>Te Anau – Fiordland at Leisure (Kepler &amp; Glowworms)</t>
         </is>
       </c>
       <c r="C151" t="inlineStr">
@@ -4837,12 +4845,12 @@
       </c>
       <c r="D151" t="inlineStr">
         <is>
-          <t>RealNZ Doubtful Sound Overnight Cruise</t>
+          <t>Te Anau Glowworm Caves Tour</t>
         </is>
       </c>
       <c r="E151" t="inlineStr">
         <is>
-          <t>https://geni.us/DoubtfulOvernight</t>
+          <t>https://geni.us/TeAnauCaves</t>
         </is>
       </c>
       <c r="F151" t="inlineStr"/>
@@ -4856,7 +4864,7 @@
       </c>
       <c r="B152" t="inlineStr">
         <is>
-          <t>Fiordland – Doubtful Sound &amp; Kepler</t>
+          <t>Te Anau – Fiordland at Leisure (Kepler &amp; Glowworms)</t>
         </is>
       </c>
       <c r="C152" t="inlineStr">
@@ -4866,12 +4874,12 @@
       </c>
       <c r="D152" t="inlineStr">
         <is>
-          <t>Te Anau Glowworm Caves Tour</t>
+          <t>Fiordland Jet</t>
         </is>
       </c>
       <c r="E152" t="inlineStr">
         <is>
-          <t>https://geni.us/TeAnauCaves</t>
+          <t>https://geni.us/FiordlandJet</t>
         </is>
       </c>
       <c r="F152" t="inlineStr"/>
@@ -4885,7 +4893,7 @@
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t>Fiordland – Doubtful Sound &amp; Kepler</t>
+          <t>Te Anau – Fiordland at Leisure (Kepler &amp; Glowworms)</t>
         </is>
       </c>
       <c r="C153" t="inlineStr">
@@ -4895,12 +4903,12 @@
       </c>
       <c r="D153" t="inlineStr">
         <is>
-          <t>Fiordland Jet</t>
+          <t>Routeburn / Key Summit Guided Walk</t>
         </is>
       </c>
       <c r="E153" t="inlineStr">
         <is>
-          <t>https://geni.us/FiordlandJet</t>
+          <t>https://geni.us/RouteburnKeyWalk</t>
         </is>
       </c>
       <c r="F153" t="inlineStr"/>
@@ -4909,27 +4917,27 @@
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t>Sat 10 Apr</t>
+          <t>Sun 11 Apr</t>
         </is>
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t>Fiordland – Doubtful Sound &amp; Kepler</t>
+          <t>Te Anau → Dunedin (Southern Scenic Route)</t>
         </is>
       </c>
       <c r="C154" t="inlineStr">
         <is>
-          <t>✨ Special Activity</t>
+          <t>🚗 Rental Car</t>
         </is>
       </c>
       <c r="D154" t="inlineStr">
         <is>
-          <t>Routeburn / Key Summit Guided Walk</t>
+          <t>Self-drive Te Anau → Dunedin via the Southern Scenic Route &amp; Catlins. The longest drive day – start early; the direct route via Gore (~3.5 hrs) is the quicker alternative.</t>
         </is>
       </c>
       <c r="E154" t="inlineStr">
         <is>
-          <t>https://geni.us/RouteburnKeyWalk</t>
+          <t>https://geni.us/RentalCarOptions</t>
         </is>
       </c>
       <c r="F154" t="inlineStr"/>
@@ -4948,17 +4956,17 @@
       </c>
       <c r="C155" t="inlineStr">
         <is>
-          <t>🚗 Rental Car</t>
+          <t>✨ Special Activity</t>
         </is>
       </c>
       <c r="D155" t="inlineStr">
         <is>
-          <t>Self-drive Te Anau → Dunedin via the Southern Scenic Route &amp; Catlins. The longest drive day – start early; the direct route via Gore (~3.5 hrs) is the quicker alternative.</t>
+          <t>Otago Peninsula Wildlife Tour (albatross &amp; penguins)</t>
         </is>
       </c>
       <c r="E155" t="inlineStr">
         <is>
-          <t>https://geni.us/RentalCarOptions</t>
+          <t>https://geni.us/DunedinWildlife</t>
         </is>
       </c>
       <c r="F155" t="inlineStr"/>
@@ -4982,12 +4990,12 @@
       </c>
       <c r="D156" t="inlineStr">
         <is>
-          <t>Otago Peninsula Wildlife Tour (albatross &amp; penguins)</t>
+          <t>Larnach Castle &amp; City Highlights Tour</t>
         </is>
       </c>
       <c r="E156" t="inlineStr">
         <is>
-          <t>https://geni.us/DunedinWildlife</t>
+          <t>https://geni.us/DunedinCityLarnach</t>
         </is>
       </c>
       <c r="F156" t="inlineStr"/>
@@ -5011,12 +5019,12 @@
       </c>
       <c r="D157" t="inlineStr">
         <is>
-          <t>Larnach Castle &amp; City Highlights Tour</t>
+          <t>Speight's Brewery Heritage Tour</t>
         </is>
       </c>
       <c r="E157" t="inlineStr">
         <is>
-          <t>https://geni.us/DunedinCityLarnach</t>
+          <t>https://geni.us/SpeightsBrewery</t>
         </is>
       </c>
       <c r="F157" t="inlineStr"/>
@@ -5040,12 +5048,12 @@
       </c>
       <c r="D158" t="inlineStr">
         <is>
-          <t>Speight's Brewery Heritage Tour</t>
+          <t>Dunedin Artisan Food Tour</t>
         </is>
       </c>
       <c r="E158" t="inlineStr">
         <is>
-          <t>https://geni.us/SpeightsBrewery</t>
+          <t>https://geni.us/ArtisanDunedin</t>
         </is>
       </c>
       <c r="F158" t="inlineStr"/>
@@ -5069,12 +5077,12 @@
       </c>
       <c r="D159" t="inlineStr">
         <is>
-          <t>Dunedin Artisan Food Tour</t>
+          <t>Olveston Historic House Tour</t>
         </is>
       </c>
       <c r="E159" t="inlineStr">
         <is>
-          <t>https://geni.us/ArtisanDunedin</t>
+          <t>https://geni.us/OlvestonHouse</t>
         </is>
       </c>
       <c r="F159" t="inlineStr"/>
@@ -5093,17 +5101,17 @@
       </c>
       <c r="C160" t="inlineStr">
         <is>
-          <t>✨ Special Activity</t>
+          <t>🏡 Accommodation (3★)</t>
         </is>
       </c>
       <c r="D160" t="inlineStr">
         <is>
-          <t>Olveston Historic House Tour</t>
+          <t>Dunedin Palms Motel</t>
         </is>
       </c>
       <c r="E160" t="inlineStr">
         <is>
-          <t>https://geni.us/OlvestonHouse</t>
+          <t>https://geni.us/DunedinPalmMotel</t>
         </is>
       </c>
       <c r="F160" t="inlineStr"/>
@@ -5122,17 +5130,17 @@
       </c>
       <c r="C161" t="inlineStr">
         <is>
-          <t>🏡 Accommodation (3★)</t>
+          <t>🏡 Accommodation (4★)</t>
         </is>
       </c>
       <c r="D161" t="inlineStr">
         <is>
-          <t>Dunedin Palms Motel</t>
+          <t>Distinction Dunedin Hotel</t>
         </is>
       </c>
       <c r="E161" t="inlineStr">
         <is>
-          <t>https://geni.us/DunedinPalmMotel</t>
+          <t>https://geni.us/DistinctionDunedin</t>
         </is>
       </c>
       <c r="F161" t="inlineStr"/>
@@ -5151,17 +5159,17 @@
       </c>
       <c r="C162" t="inlineStr">
         <is>
-          <t>🏡 Accommodation (4★)</t>
+          <t>🏡 Accommodation (5★)</t>
         </is>
       </c>
       <c r="D162" t="inlineStr">
         <is>
-          <t>Distinction Dunedin Hotel</t>
+          <t>Camp Estate, Larnach Castle</t>
         </is>
       </c>
       <c r="E162" t="inlineStr">
         <is>
-          <t>https://geni.us/DistinctionDunedin</t>
+          <t>https://geni.us/CampEstateDunedin</t>
         </is>
       </c>
       <c r="F162" t="inlineStr"/>
@@ -5170,27 +5178,27 @@
     <row r="163">
       <c r="A163" t="inlineStr">
         <is>
-          <t>Sun 11 Apr</t>
+          <t>Mon 12 Apr</t>
         </is>
       </c>
       <c r="B163" t="inlineStr">
         <is>
-          <t>Te Anau → Dunedin (Southern Scenic Route)</t>
+          <t>Dunedin &amp; Otago Peninsula</t>
         </is>
       </c>
       <c r="C163" t="inlineStr">
         <is>
-          <t>🏡 Accommodation (5★)</t>
+          <t>✨ Special Activity</t>
         </is>
       </c>
       <c r="D163" t="inlineStr">
         <is>
-          <t>Camp Estate, Larnach Castle</t>
+          <t>Otago Peninsula Wildlife Tour</t>
         </is>
       </c>
       <c r="E163" t="inlineStr">
         <is>
-          <t>https://geni.us/CampEstateDunedin</t>
+          <t>https://geni.us/DunedinWildlife</t>
         </is>
       </c>
       <c r="F163" t="inlineStr"/>
@@ -5214,12 +5222,12 @@
       </c>
       <c r="D164" t="inlineStr">
         <is>
-          <t>Otago Peninsula Wildlife Tour</t>
+          <t>Larnach Castle &amp; Gardens</t>
         </is>
       </c>
       <c r="E164" t="inlineStr">
         <is>
-          <t>https://geni.us/DunedinWildlife</t>
+          <t>https://geni.us/DunedinCityLarnach</t>
         </is>
       </c>
       <c r="F164" t="inlineStr"/>
@@ -5243,12 +5251,12 @@
       </c>
       <c r="D165" t="inlineStr">
         <is>
-          <t>Larnach Castle &amp; Gardens</t>
+          <t>Speight's Brewery Tour</t>
         </is>
       </c>
       <c r="E165" t="inlineStr">
         <is>
-          <t>https://geni.us/DunedinCityLarnach</t>
+          <t>https://geni.us/SpeightsBrewery</t>
         </is>
       </c>
       <c r="F165" t="inlineStr"/>
@@ -5272,12 +5280,12 @@
       </c>
       <c r="D166" t="inlineStr">
         <is>
-          <t>Speight's Brewery Tour</t>
+          <t>Private Dunedin Day Tour</t>
         </is>
       </c>
       <c r="E166" t="inlineStr">
         <is>
-          <t>https://geni.us/SpeightsBrewery</t>
+          <t>https://geni.us/PrivateDunedin</t>
         </is>
       </c>
       <c r="F166" t="inlineStr"/>
@@ -5286,27 +5294,27 @@
     <row r="167">
       <c r="A167" t="inlineStr">
         <is>
-          <t>Mon 12 Apr</t>
+          <t>Tue 13 Apr</t>
         </is>
       </c>
       <c r="B167" t="inlineStr">
         <is>
-          <t>Dunedin &amp; Otago Peninsula</t>
+          <t>Dunedin → Aoraki / Mount Cook (via Oamaru)</t>
         </is>
       </c>
       <c r="C167" t="inlineStr">
         <is>
-          <t>✨ Special Activity</t>
+          <t>🚗 Rental Car</t>
         </is>
       </c>
       <c r="D167" t="inlineStr">
         <is>
-          <t>Private Dunedin Day Tour</t>
+          <t>Self-drive Dunedin → Mt Cook / Mackenzie via Oamaru</t>
         </is>
       </c>
       <c r="E167" t="inlineStr">
         <is>
-          <t>https://geni.us/PrivateDunedin</t>
+          <t>https://geni.us/RentalCarOptions</t>
         </is>
       </c>
       <c r="F167" t="inlineStr"/>
@@ -5325,17 +5333,17 @@
       </c>
       <c r="C168" t="inlineStr">
         <is>
-          <t>🚗 Rental Car</t>
+          <t>✨ Special Activity</t>
         </is>
       </c>
       <c r="D168" t="inlineStr">
         <is>
-          <t>Self-drive Dunedin → Mt Cook / Mackenzie via Oamaru</t>
+          <t>Aoraki Heli-Hiking</t>
         </is>
       </c>
       <c r="E168" t="inlineStr">
         <is>
-          <t>https://geni.us/RentalCarOptions</t>
+          <t>https://geni.us/HeliHikeMtCook</t>
         </is>
       </c>
       <c r="F168" t="inlineStr"/>
@@ -5359,12 +5367,12 @@
       </c>
       <c r="D169" t="inlineStr">
         <is>
-          <t>Aoraki Heli-Hiking</t>
+          <t>Mt Cook Helicopter Flight with Snow Landing</t>
         </is>
       </c>
       <c r="E169" t="inlineStr">
         <is>
-          <t>https://geni.us/HeliHikeMtCook</t>
+          <t>https://geni.us/MtCookHeliFlight</t>
         </is>
       </c>
       <c r="F169" t="inlineStr"/>
@@ -5388,12 +5396,12 @@
       </c>
       <c r="D170" t="inlineStr">
         <is>
-          <t>Mt Cook Helicopter Flight with Snow Landing</t>
+          <t>Mt John Stargazing Experience (Tekapo)</t>
         </is>
       </c>
       <c r="E170" t="inlineStr">
         <is>
-          <t>https://geni.us/MtCookHeliFlight</t>
+          <t>https://geni.us/StargazingMtJohn</t>
         </is>
       </c>
       <c r="F170" t="inlineStr"/>
@@ -5417,12 +5425,12 @@
       </c>
       <c r="D171" t="inlineStr">
         <is>
-          <t>Mt John Stargazing Experience (Tekapo)</t>
+          <t>Dark Sky Project (Tekapo)</t>
         </is>
       </c>
       <c r="E171" t="inlineStr">
         <is>
-          <t>https://geni.us/StargazingMtJohn</t>
+          <t>https://geni.us/DarkSkyProject</t>
         </is>
       </c>
       <c r="F171" t="inlineStr"/>
@@ -5446,12 +5454,12 @@
       </c>
       <c r="D172" t="inlineStr">
         <is>
-          <t>Dark Sky Project (Tekapo)</t>
+          <t>Mt Cook / Pukaki Observatory Stargazing</t>
         </is>
       </c>
       <c r="E172" t="inlineStr">
         <is>
-          <t>https://geni.us/DarkSkyProject</t>
+          <t>https://geni.us/PukakiObservatory</t>
         </is>
       </c>
       <c r="F172" t="inlineStr"/>
@@ -5475,12 +5483,12 @@
       </c>
       <c r="D173" t="inlineStr">
         <is>
-          <t>Mt Cook / Pukaki Observatory Stargazing</t>
+          <t>Oamaru Blue Penguin Colony</t>
         </is>
       </c>
       <c r="E173" t="inlineStr">
         <is>
-          <t>https://geni.us/PukakiObservatory</t>
+          <t>https://geni.us/BluePenguinsOamaru</t>
         </is>
       </c>
       <c r="F173" t="inlineStr"/>
@@ -5499,17 +5507,17 @@
       </c>
       <c r="C174" t="inlineStr">
         <is>
-          <t>✨ Special Activity</t>
+          <t>🏡 Accommodation (3★)</t>
         </is>
       </c>
       <c r="D174" t="inlineStr">
         <is>
-          <t>Oamaru Blue Penguin Colony</t>
+          <t>Mantra Lake Tekapo</t>
         </is>
       </c>
       <c r="E174" t="inlineStr">
         <is>
-          <t>https://geni.us/BluePenguinsOamaru</t>
+          <t>https://geni.us/MantraTekapo</t>
         </is>
       </c>
       <c r="F174" t="inlineStr"/>
@@ -5528,17 +5536,17 @@
       </c>
       <c r="C175" t="inlineStr">
         <is>
-          <t>🏡 Accommodation (3★)</t>
+          <t>🏡 Accommodation (4★)</t>
         </is>
       </c>
       <c r="D175" t="inlineStr">
         <is>
-          <t>Mantra Lake Tekapo</t>
+          <t>Lakestone Lodge, Lake Pukaki</t>
         </is>
       </c>
       <c r="E175" t="inlineStr">
         <is>
-          <t>https://geni.us/MantraTekapo</t>
+          <t>https://geni.us/LakeStoneLodgePukaki</t>
         </is>
       </c>
       <c r="F175" t="inlineStr"/>
@@ -5557,17 +5565,17 @@
       </c>
       <c r="C176" t="inlineStr">
         <is>
-          <t>🏡 Accommodation (4★)</t>
+          <t>🏡 Accommodation (5★)</t>
         </is>
       </c>
       <c r="D176" t="inlineStr">
         <is>
-          <t>Lakestone Lodge, Lake Pukaki</t>
+          <t>Mt Cook Lakeview Retreat</t>
         </is>
       </c>
       <c r="E176" t="inlineStr">
         <is>
-          <t>https://geni.us/LakeStoneLodgePukaki</t>
+          <t>https://geni.us/MtCookRetreat</t>
         </is>
       </c>
       <c r="F176" t="inlineStr"/>
@@ -5586,17 +5594,17 @@
       </c>
       <c r="C177" t="inlineStr">
         <is>
-          <t>🏡 Accommodation (5★)</t>
+          <t>🏡 Accommodation (4★)</t>
         </is>
       </c>
       <c r="D177" t="inlineStr">
         <is>
-          <t>Mt Cook Lakeview Retreat</t>
+          <t>Nightsky Cottage, Twizel</t>
         </is>
       </c>
       <c r="E177" t="inlineStr">
         <is>
-          <t>https://geni.us/MtCookRetreat</t>
+          <t>https://geni.us/NightskyTwizel</t>
         </is>
       </c>
       <c r="F177" t="inlineStr"/>
@@ -5605,27 +5613,27 @@
     <row r="178">
       <c r="A178" t="inlineStr">
         <is>
-          <t>Tue 13 Apr</t>
+          <t>Wed 14 Apr</t>
         </is>
       </c>
       <c r="B178" t="inlineStr">
         <is>
-          <t>Dunedin → Aoraki / Mount Cook (via Oamaru)</t>
+          <t>Aoraki / Mount Cook National Park</t>
         </is>
       </c>
       <c r="C178" t="inlineStr">
         <is>
-          <t>🏡 Accommodation (4★)</t>
+          <t>✨ Special Activity</t>
         </is>
       </c>
       <c r="D178" t="inlineStr">
         <is>
-          <t>Nightsky Cottage, Twizel</t>
+          <t>Aoraki Heli-Hiking</t>
         </is>
       </c>
       <c r="E178" t="inlineStr">
         <is>
-          <t>https://geni.us/NightskyTwizel</t>
+          <t>https://geni.us/HeliHikeMtCook</t>
         </is>
       </c>
       <c r="F178" t="inlineStr"/>
@@ -5649,12 +5657,12 @@
       </c>
       <c r="D179" t="inlineStr">
         <is>
-          <t>Aoraki Heli-Hiking</t>
+          <t>Mt Cook Helicopter Flight with Snow Landing</t>
         </is>
       </c>
       <c r="E179" t="inlineStr">
         <is>
-          <t>https://geni.us/HeliHikeMtCook</t>
+          <t>https://geni.us/MtCookHeliFlight</t>
         </is>
       </c>
       <c r="F179" t="inlineStr"/>
@@ -5678,12 +5686,12 @@
       </c>
       <c r="D180" t="inlineStr">
         <is>
-          <t>Mt Cook Helicopter Flight with Snow Landing</t>
+          <t>Mt John Stargazing (Tekapo)</t>
         </is>
       </c>
       <c r="E180" t="inlineStr">
         <is>
-          <t>https://geni.us/MtCookHeliFlight</t>
+          <t>https://geni.us/StargazingMtJohn</t>
         </is>
       </c>
       <c r="F180" t="inlineStr"/>
@@ -5707,12 +5715,12 @@
       </c>
       <c r="D181" t="inlineStr">
         <is>
-          <t>Mt John Stargazing (Tekapo)</t>
+          <t>Mt Cook Stargazing</t>
         </is>
       </c>
       <c r="E181" t="inlineStr">
         <is>
-          <t>https://geni.us/StargazingMtJohn</t>
+          <t>https://geni.us/MtCookStargazing</t>
         </is>
       </c>
       <c r="F181" t="inlineStr"/>
@@ -5736,12 +5744,12 @@
       </c>
       <c r="D182" t="inlineStr">
         <is>
-          <t>Mt Cook Stargazing</t>
+          <t>Tekapo Scenic Flight</t>
         </is>
       </c>
       <c r="E182" t="inlineStr">
         <is>
-          <t>https://geni.us/MtCookStargazing</t>
+          <t>https://geni.us/TekapoScenicFlight</t>
         </is>
       </c>
       <c r="F182" t="inlineStr"/>
@@ -5750,27 +5758,27 @@
     <row r="183">
       <c r="A183" t="inlineStr">
         <is>
-          <t>Wed 14 Apr</t>
+          <t>Thu 15 Apr</t>
         </is>
       </c>
       <c r="B183" t="inlineStr">
         <is>
-          <t>Aoraki / Mount Cook National Park</t>
+          <t>Mount Cook → Christchurch (Inland Scenic Route)</t>
         </is>
       </c>
       <c r="C183" t="inlineStr">
         <is>
-          <t>✨ Special Activity</t>
+          <t>🚗 Rental Car</t>
         </is>
       </c>
       <c r="D183" t="inlineStr">
         <is>
-          <t>Tekapo Scenic Flight</t>
+          <t>Self-drive Mt Cook → Christchurch via the Inland Scenic Route (SH8 / SH72)</t>
         </is>
       </c>
       <c r="E183" t="inlineStr">
         <is>
-          <t>https://geni.us/TekapoScenicFlight</t>
+          <t>https://geni.us/RentalCarOptions</t>
         </is>
       </c>
       <c r="F183" t="inlineStr"/>
@@ -5789,17 +5797,17 @@
       </c>
       <c r="C184" t="inlineStr">
         <is>
-          <t>🚗 Rental Car</t>
+          <t>✨ Special Activity</t>
         </is>
       </c>
       <c r="D184" t="inlineStr">
         <is>
-          <t>Self-drive Mt Cook → Christchurch via the Inland Scenic Route (SH8 / SH72)</t>
+          <t>Christchurch Tram City Tour</t>
         </is>
       </c>
       <c r="E184" t="inlineStr">
         <is>
-          <t>https://geni.us/RentalCarOptions</t>
+          <t>https://geni.us/ChchTram</t>
         </is>
       </c>
       <c r="F184" t="inlineStr"/>
@@ -5823,12 +5831,12 @@
       </c>
       <c r="D185" t="inlineStr">
         <is>
-          <t>Christchurch Tram City Tour</t>
+          <t>Gondola, Tram &amp; Punting Combo</t>
         </is>
       </c>
       <c r="E185" t="inlineStr">
         <is>
-          <t>https://geni.us/ChchTram</t>
+          <t>https://geni.us/ChchGondolaTramPunt</t>
         </is>
       </c>
       <c r="F185" t="inlineStr"/>
@@ -5852,12 +5860,12 @@
       </c>
       <c r="D186" t="inlineStr">
         <is>
-          <t>Gondola, Tram &amp; Punting Combo</t>
+          <t>Quake City Museum</t>
         </is>
       </c>
       <c r="E186" t="inlineStr">
         <is>
-          <t>https://geni.us/ChchGondolaTramPunt</t>
+          <t>https://geni.us/ChChQuakeCity</t>
         </is>
       </c>
       <c r="F186" t="inlineStr"/>
@@ -5881,12 +5889,12 @@
       </c>
       <c r="D187" t="inlineStr">
         <is>
-          <t>Quake City Museum</t>
+          <t>Akaroa Day Tour &amp; Harbour Cruise</t>
         </is>
       </c>
       <c r="E187" t="inlineStr">
         <is>
-          <t>https://geni.us/ChChQuakeCity</t>
+          <t>https://geni.us/ChchAkaroaDayTour</t>
         </is>
       </c>
       <c r="F187" t="inlineStr"/>
@@ -5910,12 +5918,12 @@
       </c>
       <c r="D188" t="inlineStr">
         <is>
-          <t>Akaroa Day Tour &amp; Harbour Cruise</t>
+          <t>Akaroa Wildlife / Hector's Dolphin Cruise</t>
         </is>
       </c>
       <c r="E188" t="inlineStr">
         <is>
-          <t>https://geni.us/ChchAkaroaDayTour</t>
+          <t>https://geni.us/AkaroaWildlifeCruise</t>
         </is>
       </c>
       <c r="F188" t="inlineStr"/>
@@ -5939,12 +5947,12 @@
       </c>
       <c r="D189" t="inlineStr">
         <is>
-          <t>Akaroa Wildlife / Hector's Dolphin Cruise</t>
+          <t>Willowbank Wildlife Reserve</t>
         </is>
       </c>
       <c r="E189" t="inlineStr">
         <is>
-          <t>https://geni.us/AkaroaWildlifeCruise</t>
+          <t>https://geni.us/WillowbankChch</t>
         </is>
       </c>
       <c r="F189" t="inlineStr"/>
@@ -5968,12 +5976,12 @@
       </c>
       <c r="D190" t="inlineStr">
         <is>
-          <t>Willowbank Wildlife Reserve</t>
+          <t>International Antarctic Centre</t>
         </is>
       </c>
       <c r="E190" t="inlineStr">
         <is>
-          <t>https://geni.us/WillowbankChch</t>
+          <t>https://geni.us/AntarcticCentre</t>
         </is>
       </c>
       <c r="F190" t="inlineStr"/>
@@ -5992,17 +6000,17 @@
       </c>
       <c r="C191" t="inlineStr">
         <is>
-          <t>✨ Special Activity</t>
+          <t>🏡 Accommodation (3★)</t>
         </is>
       </c>
       <c r="D191" t="inlineStr">
         <is>
-          <t>International Antarctic Centre</t>
+          <t>Orari B&amp;B</t>
         </is>
       </c>
       <c r="E191" t="inlineStr">
         <is>
-          <t>https://geni.us/AntarcticCentre</t>
+          <t>https://geni.us/OrariChCh</t>
         </is>
       </c>
       <c r="F191" t="inlineStr"/>
@@ -6021,17 +6029,17 @@
       </c>
       <c r="C192" t="inlineStr">
         <is>
-          <t>🏡 Accommodation (3★)</t>
+          <t>🏡 Accommodation (4★)</t>
         </is>
       </c>
       <c r="D192" t="inlineStr">
         <is>
-          <t>Orari B&amp;B</t>
+          <t>Hotel Montreal</t>
         </is>
       </c>
       <c r="E192" t="inlineStr">
         <is>
-          <t>https://geni.us/OrariChCh</t>
+          <t>https://geni.us/HotelMontrealChch</t>
         </is>
       </c>
       <c r="F192" t="inlineStr"/>
@@ -6050,17 +6058,17 @@
       </c>
       <c r="C193" t="inlineStr">
         <is>
-          <t>🏡 Accommodation (4★)</t>
+          <t>🏡 Accommodation (5★)</t>
         </is>
       </c>
       <c r="D193" t="inlineStr">
         <is>
-          <t>Hotel Montreal</t>
+          <t>The George Hotel</t>
         </is>
       </c>
       <c r="E193" t="inlineStr">
         <is>
-          <t>https://geni.us/HotelMontrealChch</t>
+          <t>https://geni.us/TheGeorgeChCh</t>
         </is>
       </c>
       <c r="F193" t="inlineStr"/>
@@ -6079,17 +6087,17 @@
       </c>
       <c r="C194" t="inlineStr">
         <is>
-          <t>🏡 Accommodation (5★)</t>
+          <t>🏡 Accommodation (4★)</t>
         </is>
       </c>
       <c r="D194" t="inlineStr">
         <is>
-          <t>The George Hotel</t>
+          <t>Mayfair Hotel Christchurch</t>
         </is>
       </c>
       <c r="E194" t="inlineStr">
         <is>
-          <t>https://geni.us/TheGeorgeChCh</t>
+          <t>https://geni.us/MayfairChCh</t>
         </is>
       </c>
       <c r="F194" t="inlineStr"/>
@@ -6098,27 +6106,27 @@
     <row r="195">
       <c r="A195" t="inlineStr">
         <is>
-          <t>Thu 15 Apr</t>
+          <t>Fri 16 Apr</t>
         </is>
       </c>
       <c r="B195" t="inlineStr">
         <is>
-          <t>Mount Cook → Christchurch (Inland Scenic Route)</t>
+          <t>Christchurch &amp; Banks Peninsula</t>
         </is>
       </c>
       <c r="C195" t="inlineStr">
         <is>
-          <t>🏡 Accommodation (4★)</t>
+          <t>✨ Special Activity</t>
         </is>
       </c>
       <c r="D195" t="inlineStr">
         <is>
-          <t>Mayfair Hotel Christchurch</t>
+          <t>Akaroa Day Tour &amp; Harbour Cruise</t>
         </is>
       </c>
       <c r="E195" t="inlineStr">
         <is>
-          <t>https://geni.us/MayfairChCh</t>
+          <t>https://geni.us/ChchAkaroaDayTour</t>
         </is>
       </c>
       <c r="F195" t="inlineStr"/>
@@ -6142,12 +6150,12 @@
       </c>
       <c r="D196" t="inlineStr">
         <is>
-          <t>Akaroa Day Tour &amp; Harbour Cruise</t>
+          <t>Akaroa Hector's Dolphin Swim</t>
         </is>
       </c>
       <c r="E196" t="inlineStr">
         <is>
-          <t>https://geni.us/ChchAkaroaDayTour</t>
+          <t>https://geni.us/AkaroaDolphinSwim</t>
         </is>
       </c>
       <c r="F196" t="inlineStr"/>
@@ -6171,12 +6179,12 @@
       </c>
       <c r="D197" t="inlineStr">
         <is>
-          <t>Akaroa Hector's Dolphin Swim</t>
+          <t>Christchurch Gondola &amp; Tram</t>
         </is>
       </c>
       <c r="E197" t="inlineStr">
         <is>
-          <t>https://geni.us/AkaroaDolphinSwim</t>
+          <t>https://geni.us/ChchGondolaTram</t>
         </is>
       </c>
       <c r="F197" t="inlineStr"/>
@@ -6200,12 +6208,12 @@
       </c>
       <c r="D198" t="inlineStr">
         <is>
-          <t>Christchurch Gondola &amp; Tram</t>
+          <t>TranzAlpine Day Tour (Arthur's Pass)</t>
         </is>
       </c>
       <c r="E198" t="inlineStr">
         <is>
-          <t>https://geni.us/ChchGondolaTram</t>
+          <t>https://geni.us/TranzAlpDayTour</t>
         </is>
       </c>
       <c r="F198" t="inlineStr"/>
@@ -6229,12 +6237,12 @@
       </c>
       <c r="D199" t="inlineStr">
         <is>
-          <t>TranzAlpine Day Tour (Arthur's Pass)</t>
+          <t>Hot Air Balloon over Canterbury</t>
         </is>
       </c>
       <c r="E199" t="inlineStr">
         <is>
-          <t>https://geni.us/TranzAlpDayTour</t>
+          <t>https://geni.us/ChchHotAirBalloon</t>
         </is>
       </c>
       <c r="F199" t="inlineStr"/>
@@ -6243,31 +6251,35 @@
     <row r="200">
       <c r="A200" t="inlineStr">
         <is>
-          <t>Fri 16 Apr</t>
+          <t>Sat 17 Apr</t>
         </is>
       </c>
       <c r="B200" t="inlineStr">
         <is>
-          <t>Christchurch &amp; Banks Peninsula</t>
+          <t>Christchurch → Auckland → Home</t>
         </is>
       </c>
       <c r="C200" t="inlineStr">
         <is>
-          <t>✨ Special Activity</t>
+          <t>✈️ Flight</t>
         </is>
       </c>
       <c r="D200" t="inlineStr">
         <is>
-          <t>Hot Air Balloon over Canterbury</t>
+          <t>Drop rental car at Christchurch Airport · fly Christchurch → Auckland · connect to international flight home</t>
         </is>
       </c>
       <c r="E200" t="inlineStr">
         <is>
-          <t>https://geni.us/ChchHotAirBalloon</t>
+          <t>No</t>
         </is>
       </c>
       <c r="F200" t="inlineStr"/>
-      <c r="G200" t="inlineStr"/>
+      <c r="G200" t="inlineStr">
+        <is>
+          <t>Self-arranged</t>
+        </is>
+      </c>
     </row>
     <row r="201">
       <c r="A201" t="inlineStr">
@@ -6282,25 +6294,21 @@
       </c>
       <c r="C201" t="inlineStr">
         <is>
-          <t>✈️ Flight</t>
+          <t>🚖 Airport Transfer</t>
         </is>
       </c>
       <c r="D201" t="inlineStr">
         <is>
-          <t>Drop rental car at Christchurch Airport · fly Christchurch → Auckland · connect to international flight home</t>
+          <t>Airport → Christchurch → Auckland → Home</t>
         </is>
       </c>
       <c r="E201" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>https://geni.us/AirportTransfers</t>
         </is>
       </c>
       <c r="F201" t="inlineStr"/>
-      <c r="G201" t="inlineStr">
-        <is>
-          <t>Self-arranged</t>
-        </is>
-      </c>
+      <c r="G201" t="inlineStr"/>
     </row>
     <row r="202">
       <c r="A202" t="inlineStr">
@@ -6315,17 +6323,17 @@
       </c>
       <c r="C202" t="inlineStr">
         <is>
-          <t>🚖 Airport Transfer</t>
+          <t>🚗 Rental Car</t>
         </is>
       </c>
       <c r="D202" t="inlineStr">
         <is>
-          <t>Airport → Christchurch → Auckland → Home</t>
+          <t>Self-drive to Christchurch Airport (car drop) · flight CHC → AKL · international connection</t>
         </is>
       </c>
       <c r="E202" t="inlineStr">
         <is>
-          <t>https://geni.us/AirportTransfers</t>
+          <t>https://geni.us/RentalCarOptions</t>
         </is>
       </c>
       <c r="F202" t="inlineStr"/>
@@ -6344,21 +6352,25 @@
       </c>
       <c r="C203" t="inlineStr">
         <is>
-          <t>🚗 Rental Car</t>
+          <t>✈️ Flight</t>
         </is>
       </c>
       <c r="D203" t="inlineStr">
         <is>
-          <t>Self-drive to Christchurch Airport (car drop) · flight CHC → AKL · international connection</t>
+          <t>International Departure – Auckland (AKL) – Air New Zealand NZ00028 · 07:50pm</t>
         </is>
       </c>
       <c r="E203" t="inlineStr">
         <is>
-          <t>https://geni.us/RentalCarOptions</t>
+          <t>No</t>
         </is>
       </c>
       <c r="F203" t="inlineStr"/>
-      <c r="G203" t="inlineStr"/>
+      <c r="G203" t="inlineStr">
+        <is>
+          <t>Self-arranged</t>
+        </is>
+      </c>
     </row>
     <row r="204">
       <c r="A204" t="inlineStr">
@@ -6373,25 +6385,21 @@
       </c>
       <c r="C204" t="inlineStr">
         <is>
-          <t>✈️ Flight</t>
+          <t>🚖 Airport Transfer</t>
         </is>
       </c>
       <c r="D204" t="inlineStr">
         <is>
-          <t>International Departure – Auckland (AKL) – Air New Zealand NZ00028 · 07:50pm</t>
+          <t>Christchurch → Auckland → Home → Airport</t>
         </is>
       </c>
       <c r="E204" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>https://geni.us/AirportTransfers</t>
         </is>
       </c>
       <c r="F204" t="inlineStr"/>
-      <c r="G204" t="inlineStr">
-        <is>
-          <t>Self-arranged</t>
-        </is>
-      </c>
+      <c r="G204" t="inlineStr"/>
     </row>
     <row r="205">
       <c r="A205" t="inlineStr">
@@ -6406,17 +6414,17 @@
       </c>
       <c r="C205" t="inlineStr">
         <is>
-          <t>🚖 Airport Transfer</t>
+          <t>🎥 YouTube</t>
         </is>
       </c>
       <c r="D205" t="inlineStr">
         <is>
-          <t>Christchurch → Auckland → Home → Airport</t>
+          <t>NZ Trip Planning &amp; Setup</t>
         </is>
       </c>
       <c r="E205" t="inlineStr">
         <is>
-          <t>https://geni.us/AirportTransfers</t>
+          <t>https://geni.us/NZTripSetup</t>
         </is>
       </c>
       <c r="F205" t="inlineStr"/>
@@ -6440,12 +6448,12 @@
       </c>
       <c r="D206" t="inlineStr">
         <is>
-          <t>NZ Trip Planning &amp; Setup</t>
+          <t>Sample NZ Itineraries</t>
         </is>
       </c>
       <c r="E206" t="inlineStr">
         <is>
-          <t>https://geni.us/NZTripSetup</t>
+          <t>https://geni.us/NZTravelPlans</t>
         </is>
       </c>
       <c r="F206" t="inlineStr"/>
@@ -6469,12 +6477,12 @@
       </c>
       <c r="D207" t="inlineStr">
         <is>
-          <t>Sample NZ Itineraries</t>
+          <t>NZ Road Trips &amp; Scenic Drives</t>
         </is>
       </c>
       <c r="E207" t="inlineStr">
         <is>
-          <t>https://geni.us/NZTravelPlans</t>
+          <t>https://geni.us/NZRoadTrips</t>
         </is>
       </c>
       <c r="F207" t="inlineStr"/>
@@ -6498,12 +6506,12 @@
       </c>
       <c r="D208" t="inlineStr">
         <is>
-          <t>NZ Road Trips &amp; Scenic Drives</t>
+          <t>Visit Places in NZ</t>
         </is>
       </c>
       <c r="E208" t="inlineStr">
         <is>
-          <t>https://geni.us/NZRoadTrips</t>
+          <t>https://geni.us/NZVisitPlaces</t>
         </is>
       </c>
       <c r="F208" t="inlineStr"/>
@@ -6527,12 +6535,12 @@
       </c>
       <c r="D209" t="inlineStr">
         <is>
-          <t>Visit Places in NZ</t>
+          <t>Best Things To Do in NZ</t>
         </is>
       </c>
       <c r="E209" t="inlineStr">
         <is>
-          <t>https://geni.us/NZVisitPlaces</t>
+          <t>https://geni.us/NZMustDo</t>
         </is>
       </c>
       <c r="F209" t="inlineStr"/>
@@ -6556,45 +6564,16 @@
       </c>
       <c r="D210" t="inlineStr">
         <is>
-          <t>Best Things To Do in NZ</t>
+          <t>Virtual Journeys YouTube</t>
         </is>
       </c>
       <c r="E210" t="inlineStr">
         <is>
-          <t>https://geni.us/NZMustDo</t>
+          <t>https://www.youtube.com/@virtualjourneysnz</t>
         </is>
       </c>
       <c r="F210" t="inlineStr"/>
       <c r="G210" t="inlineStr"/>
-    </row>
-    <row r="211">
-      <c r="A211" t="inlineStr">
-        <is>
-          <t>Sat 17 Apr</t>
-        </is>
-      </c>
-      <c r="B211" t="inlineStr">
-        <is>
-          <t>Christchurch → Auckland → Home</t>
-        </is>
-      </c>
-      <c r="C211" t="inlineStr">
-        <is>
-          <t>🎥 YouTube</t>
-        </is>
-      </c>
-      <c r="D211" t="inlineStr">
-        <is>
-          <t>Virtual Journeys YouTube</t>
-        </is>
-      </c>
-      <c r="E211" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/@virtualjourneysnz</t>
-        </is>
-      </c>
-      <c r="F211" t="inlineStr"/>
-      <c r="G211" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>